<commit_message>
calculated timered finished algosi
</commit_message>
<xml_diff>
--- a/Курс 2 Сем 1/Алгосы/Lab21/Данные 21 алгосы.xlsx
+++ b/Курс 2 Сем 1/Алгосы/Lab21/Данные 21 алгосы.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\github\Polytech\Курс 2 Сем 1\Алгосы\Lab21\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\K\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3859AE6-EFD0-4473-83DF-F4CC8C57F791}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBF93A0D-2022-42B3-B556-80D91206C727}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="1368" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="70">
   <si>
     <t>Функция</t>
   </si>
@@ -165,9 +165,6 @@
     <t>0.000002928 сек</t>
   </si>
   <si>
-    <t>Работа с хеш таблицей (?)</t>
-  </si>
-  <si>
     <t>Пирамидальная сортировка</t>
   </si>
   <si>
@@ -187,6 +184,57 @@
   </si>
   <si>
     <t>0.080058399 сек</t>
+  </si>
+  <si>
+    <t>Хеш таблица</t>
+  </si>
+  <si>
+    <t>Поиск</t>
+  </si>
+  <si>
+    <t>0.000001251 сек</t>
+  </si>
+  <si>
+    <t>0.000003786 сек</t>
+  </si>
+  <si>
+    <t>0.000003635 сек</t>
+  </si>
+  <si>
+    <t>0.000001336 сек</t>
+  </si>
+  <si>
+    <t>0.000001993 сек</t>
+  </si>
+  <si>
+    <t>0.000024324 сек</t>
+  </si>
+  <si>
+    <t>0.000268803 сек</t>
+  </si>
+  <si>
+    <t>0.000040132 сек</t>
+  </si>
+  <si>
+    <t>0.000454548 сек</t>
+  </si>
+  <si>
+    <t>0.000602166 сек</t>
+  </si>
+  <si>
+    <t>0.062099352 сек</t>
+  </si>
+  <si>
+    <t>6.472653470 сек</t>
+  </si>
+  <si>
+    <t>0.000753802 сек</t>
+  </si>
+  <si>
+    <t>0.076900658 сек</t>
+  </si>
+  <si>
+    <t>8.219380830 сек</t>
   </si>
 </sst>
 </file>
@@ -504,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.109375" bestFit="1" customWidth="1"/>
@@ -678,36 +726,96 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>54</v>
+      </c>
+      <c r="C15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" t="s">
+        <v>60</v>
+      </c>
+      <c r="E15" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>50</v>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" t="s">
+        <v>68</v>
+      </c>
+      <c r="E20" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>